<commit_message>
data: 更新 2026-06 (TT=183.015 Kwai=58.445)
</commit_message>
<xml_diff>
--- a/docs/data/巴西数据底稿_2026-06.xlsx
+++ b/docs/data/巴西数据底稿_2026-06.xlsx
@@ -516,46 +516,46 @@
     </row>
     <row r="2">
       <c r="B2" t="n">
-        <v>339.22</v>
+        <v>434.58</v>
       </c>
       <c r="C2" t="n">
-        <v>304.29</v>
+        <v>332.03</v>
       </c>
       <c r="D2" t="n">
-        <v>1.15</v>
+        <v>1.22</v>
       </c>
       <c r="E2" t="n">
-        <v>263.1</v>
+        <v>276.84</v>
       </c>
       <c r="F2" t="n">
-        <v>9.210000000000001</v>
+        <v>10.69</v>
       </c>
       <c r="G2" t="n">
-        <v>85.48999999999999</v>
+        <v>107.45</v>
       </c>
       <c r="H2" t="n">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="I2" t="n">
-        <v>5.78</v>
+        <v>6.71</v>
       </c>
       <c r="J2" t="n">
-        <v>94.40000000000001</v>
+        <v>97.17</v>
       </c>
       <c r="K2" t="n">
-        <v>15.46</v>
+        <v>20.08</v>
       </c>
       <c r="L2" t="n">
-        <v>113.28</v>
+        <v>110.18</v>
       </c>
       <c r="M2" t="n">
-        <v>24.6</v>
+        <v>32.61</v>
       </c>
       <c r="N2" t="n">
-        <v>32.82</v>
+        <v>44.2</v>
       </c>
       <c r="O2" t="n">
-        <v>42.32</v>
+        <v>43.27</v>
       </c>
     </row>
     <row r="3">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>211.271</v>
+        <v>253.194</v>
       </c>
     </row>
     <row r="4">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>112.298</v>
+        <v>163.788</v>
       </c>
     </row>
     <row r="5">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.123</v>
+        <v>4.973</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.119</v>
+        <v>2.643</v>
       </c>
     </row>
     <row r="7">
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="9">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>60.468</v>
+        <v>88.193</v>
       </c>
     </row>
     <row r="11">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.357</v>
+        <v>2.375</v>
       </c>
     </row>
     <row r="13">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.526</v>
+        <v>0.5620000000000001</v>
       </c>
     </row>
     <row r="16">
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.281</v>
+        <v>0.297</v>
       </c>
     </row>
     <row r="17">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.242</v>
+        <v>0.257</v>
       </c>
     </row>
     <row r="18">
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.099</v>
+        <v>0.104</v>
       </c>
     </row>
     <row r="20">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>232.337</v>
+        <v>242.989</v>
       </c>
     </row>
     <row r="21">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>11.393</v>
+        <v>13.616</v>
       </c>
     </row>
     <row r="22">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>4.029</v>
+        <v>3.884</v>
       </c>
     </row>
     <row r="23">
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2.814</v>
+        <v>2.838</v>
       </c>
     </row>
     <row r="24">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>2.317</v>
+        <v>2.705</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.836</v>
+        <v>4.725</v>
       </c>
     </row>
     <row r="27">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.231</v>
+        <v>2.576</v>
       </c>
     </row>
     <row r="28">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.302</v>
+        <v>1.279</v>
       </c>
     </row>
     <row r="29">
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.838</v>
+        <v>0.827</v>
       </c>
     </row>
     <row r="30">
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.446</v>
+        <v>0.538</v>
       </c>
     </row>
     <row r="32">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>61.823</v>
+        <v>81.40600000000001</v>
       </c>
     </row>
     <row r="33">
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>8.978999999999999</v>
+        <v>10.687</v>
       </c>
     </row>
     <row r="34">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>5.715</v>
+        <v>5.836</v>
       </c>
     </row>
     <row r="35">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>5.662</v>
+        <v>5.789</v>
       </c>
     </row>
     <row r="36">
@@ -845,57 +845,57 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1.697</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Google News</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>0.075</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Panflix</t>
+          <t>Google News</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>0.073</v>
+        <v>0.08699999999999999</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>Panflix</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>0.065</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Estadao</t>
+          <t>UOL | Notícias em Tempo Real</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>UOL | Notícias em Tempo Real</t>
+          <t>Zero Hora</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>0.033</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="44">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="I44" t="n">
-        <v>1.415</v>
+        <v>1.714</v>
       </c>
     </row>
     <row r="45">
@@ -915,37 +915,37 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.746</v>
+        <v>0.762</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ReadEra by READERA LLC</t>
+          <t>Kindle</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.436</v>
+        <v>0.502</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Webnovel</t>
+          <t>ReadEra by READERA LLC</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>0.338</v>
+        <v>0.416</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kindle</t>
+          <t>Webnovel</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>0.272</v>
+        <v>0.339</v>
       </c>
     </row>
     <row r="50">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>57.742</v>
+        <v>57.436</v>
       </c>
     </row>
     <row r="51">
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>23.271</v>
+        <v>26.78</v>
       </c>
     </row>
     <row r="52">
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>3.674</v>
+        <v>3.583</v>
       </c>
     </row>
     <row r="53">
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>2.565</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="54">
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>1.945</v>
+        <v>1.836</v>
       </c>
     </row>
     <row r="56">
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>5.527</v>
+        <v>9.484999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -1015,7 +1015,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>4.564</v>
+        <v>4.817</v>
       </c>
     </row>
     <row r="58">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>0.978</v>
+        <v>0.969</v>
       </c>
     </row>
     <row r="59">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>0.659</v>
+        <v>0.637</v>
       </c>
     </row>
     <row r="60">
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="L62" t="n">
-        <v>35.569</v>
+        <v>31.119</v>
       </c>
     </row>
     <row r="63">
@@ -1065,27 +1065,27 @@
         </is>
       </c>
       <c r="L63" t="n">
-        <v>5.193</v>
+        <v>4.948</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Minecraft Pocket Edition</t>
+          <t>Free Fire</t>
         </is>
       </c>
       <c r="L64" t="n">
-        <v>4.456</v>
+        <v>4.56</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Free Fire</t>
+          <t>Minecraft Pocket Edition</t>
         </is>
       </c>
       <c r="L65" t="n">
-        <v>4.358</v>
+        <v>3.937</v>
       </c>
     </row>
     <row r="66">
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="L66" t="n">
-        <v>2.075</v>
+        <v>2.294</v>
       </c>
     </row>
     <row r="68">
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>10.824</v>
+        <v>15.118</v>
       </c>
     </row>
     <row r="69">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>5.795</v>
+        <v>7.282</v>
       </c>
     </row>
     <row r="70">
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>2.516</v>
+        <v>3.418</v>
       </c>
     </row>
     <row r="71">
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>1.132</v>
+        <v>1.483</v>
       </c>
     </row>
     <row r="72">
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="M72" t="n">
-        <v>0.923</v>
+        <v>1.036</v>
       </c>
     </row>
     <row r="74">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>4.639</v>
+        <v>9.010999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -1165,37 +1165,37 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>3.926</v>
+        <v>4.599</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Uber Driver</t>
+          <t>99 POP</t>
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2.708</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>99 POP</t>
+          <t>Nubank</t>
         </is>
       </c>
       <c r="N77" t="n">
-        <v>2.657</v>
+        <v>3.005</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Nubank</t>
+          <t>99Taxis</t>
         </is>
       </c>
       <c r="N78" t="n">
-        <v>2.417</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="80">
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="O80" t="n">
-        <v>13.275</v>
+        <v>14.132</v>
       </c>
     </row>
     <row r="81">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="O81" t="n">
-        <v>10.106</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="82">
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="O82" t="n">
-        <v>6.701</v>
+        <v>6.505</v>
       </c>
     </row>
     <row r="83">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="O83" t="n">
-        <v>2.659</v>
+        <v>2.533</v>
       </c>
     </row>
     <row r="84">
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="O84" t="n">
-        <v>2.127</v>
+        <v>2.009</v>
       </c>
     </row>
     <row r="86">
@@ -1255,40 +1255,40 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>7.602</v>
+        <v>8.186</v>
       </c>
       <c r="E86" t="n">
-        <v>10.21</v>
+        <v>10.805</v>
       </c>
       <c r="F86" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.742</v>
       </c>
       <c r="G86" t="n">
-        <v>1.619</v>
+        <v>1.793</v>
       </c>
       <c r="H86" t="n">
-        <v>0.165</v>
+        <v>0.222</v>
       </c>
       <c r="I86" t="n">
-        <v>2.571</v>
+        <v>2.975</v>
       </c>
       <c r="J86" t="n">
-        <v>5.199</v>
+        <v>5.12</v>
       </c>
       <c r="K86" t="n">
-        <v>3.486</v>
+        <v>3.929</v>
       </c>
       <c r="L86" t="n">
-        <v>61.628</v>
+        <v>63.322</v>
       </c>
       <c r="M86" t="n">
-        <v>3.412</v>
+        <v>4.273</v>
       </c>
       <c r="N86" t="n">
-        <v>16.476</v>
+        <v>21.378</v>
       </c>
       <c r="O86" t="n">
-        <v>7.45</v>
+        <v>7.541</v>
       </c>
     </row>
   </sheetData>

</xml_diff>